<commit_message>
Add JTBD job statements to sub-job rows in GitOps draft working sheet
Updated 18 rows in the "Mapping existing content to jobs" sheet to include
proper JTBD-formatted job statements following the "When [situation], I want
to [action], so I can [outcome]" pattern. This ensures all sub-job entries
have user-centered job statements rather than simple task descriptions.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/GitOps draft working sheet.xlsx
+++ b/analysis/GitOps draft working sheet.xlsx
@@ -14101,7 +14101,7 @@
       <c r="B7" s="18" t="n"/>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Size Redis resources for large-scale deployments</t>
+          <t>When planning a large-scale GitOps deployment, I want to size Redis resources appropriately, so I can ensure optimal performance and avoid resource constraints</t>
         </is>
       </c>
       <c r="D7" s="18" t="n"/>
@@ -14116,7 +14116,7 @@
       <c r="B8" s="18" t="n"/>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Understand resource requirements for default GitOps workloads</t>
+          <t>When planning my GitOps deployment, I want to understand resource requirements for default workloads, so I can allocate sufficient cluster capacity</t>
         </is>
       </c>
       <c r="D8" s="18" t="n"/>
@@ -14337,7 +14337,7 @@
       <c r="B22" s="18" t="n"/>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Complete installation and verify deployment</t>
+          <t>When installing the GitOps Operator, I want to complete the installation and verify deployment, so I can confirm the system is running correctly</t>
         </is>
       </c>
       <c r="D22" s="18" t="n"/>
@@ -14352,7 +14352,7 @@
       <c r="B23" s="18" t="n"/>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Configure Operator installation settings</t>
+          <t>When installing the GitOps Operator, I want to configure installation settings, so I can customize the deployment to my requirements</t>
         </is>
       </c>
       <c r="D23" s="18" t="n"/>
@@ -14367,7 +14367,7 @@
       <c r="B24" s="18" t="n"/>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Create and apply OperatorGroup</t>
+          <t>When installing the GitOps Operator, I want to create and apply an OperatorGroup, so I can define the Operator's target namespaces</t>
         </is>
       </c>
       <c r="D24" s="18" t="n"/>
@@ -14382,7 +14382,7 @@
       <c r="B25" s="18" t="n"/>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Create and configure Operator namespace</t>
+          <t>When installing the GitOps Operator, I want to create and configure the Operator namespace, so I can isolate GitOps resources</t>
         </is>
       </c>
       <c r="D25" s="18" t="n"/>
@@ -14397,7 +14397,7 @@
       <c r="B26" s="18" t="n"/>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>Download and extract CLI archive</t>
+          <t>When installing the GitOps CLI, I want to download and extract the CLI archive, so I can prepare the binary for installation</t>
         </is>
       </c>
       <c r="D26" s="18" t="n"/>
@@ -14412,7 +14412,7 @@
       <c r="B27" s="18" t="n"/>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>Install CLI binary to PATH</t>
+          <t>When installing the GitOps CLI, I want to install the CLI binary to my PATH, so I can run GitOps commands from any directory</t>
         </is>
       </c>
       <c r="D27" s="18" t="n"/>
@@ -14427,7 +14427,7 @@
       <c r="B28" s="18" t="n"/>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>Install CLI to PATH</t>
+          <t>When installing the GitOps CLI, I want to install the CLI to my PATH, so I can access GitOps commands system-wide</t>
         </is>
       </c>
       <c r="D28" s="18" t="n"/>
@@ -14442,7 +14442,7 @@
       <c r="B29" s="18" t="n"/>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Install and verify CLI package</t>
+          <t>When installing the GitOps CLI via RPM, I want to install and verify the CLI package, so I can ensure the installation was successful</t>
         </is>
       </c>
       <c r="D29" s="18" t="n"/>
@@ -14457,7 +14457,7 @@
       <c r="B30" s="18" t="n"/>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>Navigate to OperatorHub and locate GitOps Operator</t>
+          <t>When installing the GitOps Operator via web console, I want to navigate to OperatorHub and locate the GitOps Operator, so I can begin the installation process</t>
         </is>
       </c>
       <c r="D30" s="18" t="n"/>
@@ -14472,7 +14472,7 @@
       <c r="B31" s="18" t="n"/>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>Register system and enable GitOps repositories</t>
+          <t>When installing the GitOps CLI via RPM, I want to register my system and enable GitOps repositories, so I can access the GitOps packages</t>
         </is>
       </c>
       <c r="D31" s="18" t="n"/>
@@ -14487,7 +14487,7 @@
       <c r="B32" s="18" t="n"/>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>Subscribe namespace to GitOps Operator</t>
+          <t>When installing the GitOps Operator, I want to subscribe my namespace to the GitOps Operator, so I can enable GitOps functionality</t>
         </is>
       </c>
       <c r="D32" s="18" t="n"/>
@@ -14502,7 +14502,7 @@
       <c r="B33" s="18" t="n"/>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>Verify CLI installation</t>
+          <t>When installing the GitOps CLI, I want to verify the CLI installation, so I can confirm it's working correctly</t>
         </is>
       </c>
       <c r="D33" s="18" t="n"/>
@@ -14517,7 +14517,7 @@
       <c r="B34" s="18" t="n"/>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>Verify GitOps pod deployment</t>
+          <t>When installing the GitOps Operator, I want to verify GitOps pod deployment, so I can confirm the Operator is running successfully</t>
         </is>
       </c>
       <c r="D34" s="18" t="n"/>
@@ -14632,7 +14632,7 @@
       <c r="B42" s="18" t="n"/>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Authenticate with OpenShift credentials</t>
+          <t>When accessing the Argo CD instance, I want to authenticate with my OpenShift credentials, so I can use my existing cluster identity</t>
         </is>
       </c>
       <c r="D42" s="18" t="n"/>
@@ -14647,7 +14647,7 @@
       <c r="B43" s="18" t="n"/>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Authenticate with admin credentials</t>
+          <t>When accessing the Argo CD instance, I want to authenticate with admin credentials, so I can perform administrative tasks</t>
         </is>
       </c>
       <c r="D43" s="18" t="n"/>
@@ -14662,7 +14662,7 @@
       <c r="B44" s="18" t="n"/>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Navigate to Argo CD UI</t>
+          <t>When accessing the Argo CD instance, I want to navigate to the Argo CD UI, so I can manage my GitOps deployments visually</t>
         </is>
       </c>
       <c r="D44" s="18" t="n"/>

</xml_diff>